<commit_message>
BOM update, new relay + new P side mosfet + Aliexpress links and price
</commit_message>
<xml_diff>
--- a/BOM_LignePassionIIm.xlsx
+++ b/BOM_LignePassionIIm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79fc430203973324/TravauxMetriques/IIm/Passion IIm/PupitreLigne/AlimLigne_PassionIIm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a43dc3239fed0de/PCB_Perso/PCB_IIm_Ligne/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="325" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{554F8893-E192-42BB-B486-75A96D8534B9}"/>
+  <xr:revisionPtr revIDLastSave="348" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FC5694C-C4FF-4997-9199-556382D8D3CF}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
   <si>
     <t>Quoi</t>
   </si>
@@ -90,21 +90,12 @@
     <t>Relai BiStable de Puissance</t>
   </si>
   <si>
-    <t>Omron</t>
-  </si>
-  <si>
     <t>Digikey</t>
   </si>
   <si>
-    <t>https://www.digikey.ch/fr/products/detail/omron-electronics-inc-emc-div/G2RK-2-DC12/259703</t>
-  </si>
-  <si>
     <t>Relai Bistable de Signal</t>
   </si>
   <si>
-    <t>MPSA56</t>
-  </si>
-  <si>
     <t>Ref PCB</t>
   </si>
   <si>
@@ -150,9 +141,6 @@
     <t>https://www.digikey.ch/fr/products/detail/diotec-semiconductor/1N4007/18833652</t>
   </si>
   <si>
-    <t>https://www.digikey.ch/fr/products/detail/diotec-semiconductor/MPSA56/22193185</t>
-  </si>
-  <si>
     <t>BOM - PCB Bloc de Ligne Passion IIM</t>
   </si>
   <si>
@@ -346,6 +334,27 @@
   </si>
   <si>
     <t>~1000uF</t>
+  </si>
+  <si>
+    <t>Finder</t>
+  </si>
+  <si>
+    <t>https://www.conrad.ch/fr/p/finder-41-52-6-012-4016-relais-pour-circuits-imprimes-12-v-dc-8-a-2-inverseurs-rt-1-pc-s-1419696.html</t>
+  </si>
+  <si>
+    <t>Impression 3D</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005012410174447.html?spm=a2g0o.productlist.main.3.1c57pPLrpPLrXF&amp;algo_pvid=8d846d87-e1c7-4911-9404-42bf57029f2f&amp;pdp_ext_f=%7B%22order%22%3A%223%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005012410174447%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005008777027854.html?spm=a2g0o.productlist.main.3.34a9f054Jnh2d5&amp;algo_pvid=a3217470-cd61-4707-8b2f-7d76497918d0&amp;pdp_ext_f=%7B%22order%22%3A%221295%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005008777027854%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>IRFU5305PBF</t>
+  </si>
+  <si>
+    <t>https://www.conrad.ch/fr/p/infineon-technologies-irfu5305pbf-mosfet-1-canal-p-110-w-i-pak-162729.html?insert=UP</t>
   </si>
 </sst>
 </file>
@@ -355,7 +364,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;CHF&quot;_-;\-* #,##0.00\ &quot;CHF&quot;_-;_-* &quot;-&quot;??\ &quot;CHF&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -382,6 +391,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -526,11 +543,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -563,6 +581,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -590,12 +609,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -614,24 +653,6 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;CHF&quot;_-;\-* #,##0.00\ &quot;CHF&quot;_-;_-* &quot;-&quot;??\ &quot;CHF&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -750,10 +771,10 @@
     <tableColumn id="5" xr3:uid="{99AE4783-A1AE-4A59-8D0A-2F21D4650621}" name="Qty/PCB"/>
     <tableColumn id="6" xr3:uid="{7DFEF622-3863-4E1B-9C42-44C137F57007}" name="Qty/Tot"/>
     <tableColumn id="7" xr3:uid="{395CF200-6735-4436-81FB-32A22C5D952F}" name="Prix" dataDxfId="2" dataCellStyle="Monétaire"/>
-    <tableColumn id="8" xr3:uid="{AF9D19B1-93B1-4ACE-B10F-818FD3288CA4}" name="PrixTot/PCB" dataDxfId="0" dataCellStyle="Monétaire">
+    <tableColumn id="8" xr3:uid="{AF9D19B1-93B1-4ACE-B10F-818FD3288CA4}" name="PrixTot/PCB" dataDxfId="1" dataCellStyle="Monétaire">
       <calculatedColumnFormula>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B4254C8A-C5D7-4572-B86E-606DB6474104}" name="Fabriquant" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{B4254C8A-C5D7-4572-B86E-606DB6474104}" name="Fabriquant" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{CF25DBB4-03E2-4519-889D-8135C83E9E6E}" name="Fournisseur "/>
     <tableColumn id="11" xr3:uid="{BD2CA350-D119-422A-BE3F-FA523F34F5B9}" name="Lien "/>
   </tableColumns>
@@ -1079,47 +1100,47 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B7EC6F-57FE-4577-A1D4-89717E48955F}">
   <dimension ref="A1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" customWidth="1"/>
-    <col min="10" max="10" width="19.88671875" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" customWidth="1"/>
-    <col min="12" max="12" width="79.5546875" customWidth="1"/>
+    <col min="1" max="1" width="25.53125" customWidth="1"/>
+    <col min="2" max="2" width="18.1328125" customWidth="1"/>
+    <col min="3" max="3" width="12.796875" customWidth="1"/>
+    <col min="4" max="4" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.86328125" customWidth="1"/>
+    <col min="9" max="9" width="12.1328125" customWidth="1"/>
+    <col min="10" max="10" width="19.86328125" customWidth="1"/>
+    <col min="11" max="11" width="12.46484375" customWidth="1"/>
+    <col min="12" max="12" width="79.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-    </row>
-    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+    </row>
+    <row r="2" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>1</v>
@@ -1134,7 +1155,7 @@
         <v>4</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J2" s="12" t="s">
         <v>5</v>
@@ -1146,12 +1167,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -1159,29 +1180,29 @@
       <c r="F3">
         <v>1</v>
       </c>
-      <c r="H3" s="2">
-        <v>8.7200000000000006</v>
+      <c r="H3" s="24">
+        <v>5.5</v>
       </c>
       <c r="I3" s="2">
         <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
-        <v>8.7200000000000006</v>
+        <v>5.5</v>
       </c>
       <c r="J3" t="s">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="K3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="L3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1194,18 +1215,18 @@
         <v>0.5</v>
       </c>
       <c r="K4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>555</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1218,55 +1239,55 @@
         <v>0.68</v>
       </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="H6" s="2">
-        <v>0.11</v>
+        <v>0.42</v>
       </c>
       <c r="I6" s="2">
         <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
-        <v>0.11</v>
+        <v>0.42</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="K6" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -1279,24 +1300,24 @@
         <v>0.255</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -1309,24 +1330,24 @@
         <v>2.48</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="K8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -1338,15 +1359,15 @@
       </c>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -1360,18 +1381,18 @@
       </c>
       <c r="J10" s="4"/>
       <c r="K10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -1385,18 +1406,18 @@
       </c>
       <c r="J11" s="4"/>
       <c r="K11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -1408,16 +1429,16 @@
       </c>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F13">
         <v>4</v>
@@ -1430,24 +1451,24 @@
         <v>0.27200000000000002</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F14">
         <v>3</v>
@@ -1459,18 +1480,18 @@
       </c>
       <c r="J14" s="4"/>
       <c r="K14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1481,18 +1502,18 @@
         <v>0</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F16">
         <v>5</v>
@@ -1506,18 +1527,18 @@
       </c>
       <c r="J16" s="4"/>
       <c r="K16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -1531,18 +1552,18 @@
       </c>
       <c r="J17" s="4"/>
       <c r="K17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -1556,18 +1577,18 @@
       </c>
       <c r="J18" s="4"/>
       <c r="K18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F19">
         <v>2</v>
@@ -1581,15 +1602,15 @@
       </c>
       <c r="J19" s="4"/>
       <c r="K19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D20" s="3"/>
       <c r="F20">
@@ -1603,18 +1624,18 @@
         <v>0.05</v>
       </c>
       <c r="K20" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F21">
         <v>4</v>
@@ -1627,12 +1648,12 @@
         <v>0.2</v>
       </c>
       <c r="K21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F22">
         <v>2</v>
@@ -1646,15 +1667,15 @@
       </c>
       <c r="J22" s="4"/>
       <c r="K22" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="L22" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -1668,15 +1689,15 @@
       </c>
       <c r="J23" s="4"/>
       <c r="K23" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -1690,15 +1711,15 @@
       </c>
       <c r="J24" s="4"/>
       <c r="K24" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L24" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -1712,15 +1733,15 @@
       </c>
       <c r="J25" s="4"/>
       <c r="K25" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L25" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -1734,18 +1755,18 @@
       </c>
       <c r="J26" s="4"/>
       <c r="K26" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F27">
         <v>1</v>
@@ -1759,69 +1780,84 @@
       </c>
       <c r="J27" s="4"/>
       <c r="K27" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="L27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2">
+        <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
+        <v>1</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" t="s">
         <v>94</v>
       </c>
-      <c r="F28">
-        <v>1</v>
-      </c>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2">
-        <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="4"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D29" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2">
+        <v>1.52</v>
+      </c>
       <c r="I29" s="2">
         <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
-        <v>0</v>
+        <v>1.52</v>
       </c>
       <c r="J29" s="4"/>
       <c r="K29" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F30">
         <v>2</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="H30" s="2">
+        <v>0.43</v>
+      </c>
       <c r="I30" s="2">
         <f>Tableau2[[#This Row],[Qty/PCB]]*Tableau2[[#This Row],[Prix]]</f>
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="J30" s="4"/>
       <c r="K30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L30" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D31" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F31">
         <v>2</v>
@@ -1835,15 +1871,15 @@
       </c>
       <c r="J31" s="4"/>
       <c r="K31" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D32" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F32">
         <v>2</v>
@@ -1857,76 +1893,76 @@
       </c>
       <c r="J32" s="4"/>
       <c r="K32" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="8">
         <v>46126</v>
       </c>
-      <c r="D34" s="15" t="e" vm="1">
+      <c r="D34" s="16" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="E34" s="16"/>
-      <c r="F34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="18"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" s="7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D35" s="18"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="19"/>
+        <v>28</v>
+      </c>
+      <c r="D35" s="19"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="20"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" s="7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D36" s="18"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="19"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="20"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="20"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="22"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="D37" s="21"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="23"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
@@ -1935,10 +1971,13 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="D34:F37"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="L3" r:id="rId1" xr:uid="{B3065FAB-E838-4A51-A82F-630335C42D81}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>